<commit_message>
Stop collecting from Manchester
- Allowed collection cities: London, Birmingham, Leeds.
- Hints, chat questions and samples no longer mention Manchester
  (the template's example row BK-001 stays as-is so uploads still skip it).
- Regenerated sample sheets; test that Manchester is refused.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/planted-mistakes.xlsx
+++ b/samples/planted-mistakes.xlsx
@@ -924,7 +924,7 @@
         <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
         <v>44</v>
@@ -1190,7 +1190,7 @@
         <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
         <v>38</v>

</xml_diff>